<commit_message>
docs: align handoff dates and test prerequisites in WBS
</commit_message>
<xml_diff>
--- a/plans/wbs/otter-shield-wbs-final.xlsx
+++ b/plans/wbs/otter-shield-wbs-final.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="게시용 1-39" sheetId="1" r:id="R526bae6381da4f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="게시용 40-73" sheetId="2" r:id="Rd45ba8a368eb402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상세실행" sheetId="3" r:id="R8f6a21c5d3724828"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변경·인계" sheetId="4" r:id="Re108d49fbacd469c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M5 시간계획" sheetId="5" r:id="R78c0165d754e4c76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="게시용 1-39" sheetId="1" r:id="Rcae57fce70ac4122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="게시용 40-73" sheetId="2" r:id="R8db0252826384566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상세실행" sheetId="3" r:id="Ra6fec01c64234159"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변경·인계" sheetId="4" r:id="Rc6fa07c5508843f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M5 시간계획" sheetId="5" r:id="R7649f3accf6b4237"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -121,7 +121,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -208,6 +208,21 @@
         <x:fgColor rgb="FFFFF4D8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEDE9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE1ECDD"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border>
@@ -290,7 +305,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="99">
+  <x:cellXfs count="105">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -540,6 +555,24 @@
     <x:xf numFmtId="202" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="17" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="17" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -551,7 +584,7 @@
         <x:color rgb="FF9A302B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE1DF"/>
         </x:patternFill>
       </x:fill>
@@ -561,7 +594,7 @@
         <x:color rgb="FF805A1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D5"/>
         </x:patternFill>
       </x:fill>
@@ -572,7 +605,7 @@
         <x:color rgb="FF9A302B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE1DF"/>
         </x:patternFill>
       </x:fill>
@@ -3351,40 +3384,40 @@
         <x:v>M3 홍은서</x:v>
       </x:c>
       <x:c r="D8" s="50" t="n">
-        <x:v>46330</x:v>
+        <x:v>46331</x:v>
       </x:c>
       <x:c r="E8" s="49" t="str">
         <x:v>미확인</x:v>
       </x:c>
-      <x:c r="F8" s="29"/>
-      <x:c r="G8" s="29"/>
-      <x:c r="H8" s="29"/>
-      <x:c r="I8" s="29"/>
-      <x:c r="J8" s="29"/>
-      <x:c r="K8" s="33"/>
-      <x:c r="L8" s="33"/>
-      <x:c r="M8" s="29"/>
-      <x:c r="N8" s="29"/>
-      <x:c r="O8" s="29"/>
-      <x:c r="P8" s="29"/>
-      <x:c r="Q8" s="29"/>
-      <x:c r="R8" s="33"/>
-      <x:c r="S8" s="33"/>
-      <x:c r="T8" s="29"/>
-      <x:c r="U8" s="29"/>
-      <x:c r="V8" s="31"/>
-      <x:c r="W8" s="29"/>
-      <x:c r="X8" s="29"/>
-      <x:c r="Y8" s="33"/>
-      <x:c r="Z8" s="33"/>
-      <x:c r="AA8" s="29"/>
-      <x:c r="AB8" s="29"/>
-      <x:c r="AC8" s="29"/>
-      <x:c r="AD8" s="29"/>
-      <x:c r="AE8" s="29"/>
-      <x:c r="AF8" s="33"/>
-      <x:c r="AG8" s="33"/>
-      <x:c r="AH8" s="29"/>
+      <x:c r="F8" s="99"/>
+      <x:c r="G8" s="99"/>
+      <x:c r="H8" s="99"/>
+      <x:c r="I8" s="99"/>
+      <x:c r="J8" s="99"/>
+      <x:c r="K8" s="99"/>
+      <x:c r="L8" s="99"/>
+      <x:c r="M8" s="99"/>
+      <x:c r="N8" s="99"/>
+      <x:c r="O8" s="99"/>
+      <x:c r="P8" s="99"/>
+      <x:c r="Q8" s="99"/>
+      <x:c r="R8" s="99"/>
+      <x:c r="S8" s="99"/>
+      <x:c r="T8" s="99"/>
+      <x:c r="U8" s="99"/>
+      <x:c r="V8" s="101"/>
+      <x:c r="W8" s="102"/>
+      <x:c r="X8" s="99"/>
+      <x:c r="Y8" s="99"/>
+      <x:c r="Z8" s="99"/>
+      <x:c r="AA8" s="99"/>
+      <x:c r="AB8" s="99"/>
+      <x:c r="AC8" s="99"/>
+      <x:c r="AD8" s="99"/>
+      <x:c r="AE8" s="99"/>
+      <x:c r="AF8" s="99"/>
+      <x:c r="AG8" s="99"/>
+      <x:c r="AH8" s="99"/>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
       <x:c r="A9" s="38" t="str">
@@ -3397,40 +3430,40 @@
         <x:v>M4 박진혁</x:v>
       </x:c>
       <x:c r="D9" s="51" t="n">
-        <x:v>46330</x:v>
+        <x:v>46331</x:v>
       </x:c>
       <x:c r="E9" s="48" t="str">
         <x:v>미확인</x:v>
       </x:c>
-      <x:c r="F9" s="29"/>
-      <x:c r="G9" s="29"/>
-      <x:c r="H9" s="29"/>
-      <x:c r="I9" s="29"/>
-      <x:c r="J9" s="29"/>
-      <x:c r="K9" s="33"/>
-      <x:c r="L9" s="33"/>
-      <x:c r="M9" s="29"/>
-      <x:c r="N9" s="29"/>
-      <x:c r="O9" s="29"/>
-      <x:c r="P9" s="29"/>
-      <x:c r="Q9" s="29"/>
-      <x:c r="R9" s="33"/>
-      <x:c r="S9" s="33"/>
-      <x:c r="T9" s="29"/>
-      <x:c r="U9" s="29"/>
-      <x:c r="V9" s="31"/>
-      <x:c r="W9" s="29"/>
-      <x:c r="X9" s="29"/>
-      <x:c r="Y9" s="33"/>
-      <x:c r="Z9" s="33"/>
-      <x:c r="AA9" s="29"/>
-      <x:c r="AB9" s="29"/>
-      <x:c r="AC9" s="29"/>
-      <x:c r="AD9" s="29"/>
-      <x:c r="AE9" s="29"/>
-      <x:c r="AF9" s="33"/>
-      <x:c r="AG9" s="33"/>
-      <x:c r="AH9" s="29"/>
+      <x:c r="F9" s="99"/>
+      <x:c r="G9" s="99"/>
+      <x:c r="H9" s="99"/>
+      <x:c r="I9" s="99"/>
+      <x:c r="J9" s="99"/>
+      <x:c r="K9" s="99"/>
+      <x:c r="L9" s="99"/>
+      <x:c r="M9" s="99"/>
+      <x:c r="N9" s="99"/>
+      <x:c r="O9" s="99"/>
+      <x:c r="P9" s="99"/>
+      <x:c r="Q9" s="99"/>
+      <x:c r="R9" s="99"/>
+      <x:c r="S9" s="99"/>
+      <x:c r="T9" s="99"/>
+      <x:c r="U9" s="99"/>
+      <x:c r="V9" s="103"/>
+      <x:c r="W9" s="104"/>
+      <x:c r="X9" s="99"/>
+      <x:c r="Y9" s="99"/>
+      <x:c r="Z9" s="99"/>
+      <x:c r="AA9" s="99"/>
+      <x:c r="AB9" s="99"/>
+      <x:c r="AC9" s="99"/>
+      <x:c r="AD9" s="99"/>
+      <x:c r="AE9" s="99"/>
+      <x:c r="AF9" s="99"/>
+      <x:c r="AG9" s="99"/>
+      <x:c r="AH9" s="99"/>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
       <x:c r="A10" s="21" t="str">
@@ -5110,7 +5143,7 @@
         <x:v>M1 주관·전원</x:v>
       </x:c>
       <x:c r="E9" s="75" t="n">
-        <x:v>46323</x:v>
+        <x:v>46324</x:v>
       </x:c>
       <x:c r="F9" s="75" t="n">
         <x:v>46324</x:v>
@@ -5245,7 +5278,7 @@
         <x:v>미확인</x:v>
       </x:c>
       <x:c r="L12" s="74" t="str">
-        <x:v>실측 잔여 작업 시간로 11/06 이후 기능 추가 여부 결정</x:v>
+        <x:v>남은 작업의 예상 소요 시간으로 11/06 이후 기능 추가 여부 결정</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="70" customHeight="1">
@@ -6440,7 +6473,7 @@
         <x:v>M2 윤서영</x:v>
       </x:c>
       <x:c r="E44" s="75" t="n">
-        <x:v>46324</x:v>
+        <x:v>46325</x:v>
       </x:c>
       <x:c r="F44" s="75" t="n">
         <x:v>46325</x:v>
@@ -6972,7 +7005,7 @@
         <x:v>M3 홍은서</x:v>
       </x:c>
       <x:c r="E58" s="75" t="n">
-        <x:v>46323</x:v>
+        <x:v>46324</x:v>
       </x:c>
       <x:c r="F58" s="75" t="n">
         <x:v>46324</x:v>
@@ -7314,7 +7347,7 @@
         <x:v>M4 박진혁</x:v>
       </x:c>
       <x:c r="E67" s="75" t="n">
-        <x:v>46322</x:v>
+        <x:v>46323</x:v>
       </x:c>
       <x:c r="F67" s="75" t="n">
         <x:v>46323</x:v>
@@ -8042,7 +8075,7 @@
         <x:v>46325</x:v>
       </x:c>
       <x:c r="G86" s="74" t="str">
-        <x:v>M5-A03, M5-A04, M1-A15, DEV03</x:v>
+        <x:v>M5-A03, M5-A04, M1-A15, DEV03, M1-A16</x:v>
       </x:c>
       <x:c r="H86" s="74" t="str">
         <x:v>캐나다→한국 정상 업무·Test DB 시험 준비</x:v>
@@ -8057,7 +8090,7 @@
         <x:v>미확인</x:v>
       </x:c>
       <x:c r="L86" s="74" t="str">
-        <x:v>실제 공격 기록은 11/02</x:v>
+        <x:v>M1 게시판 배포 완료 후 캐나다에서 정상 접속 확인. Test DB 경로는 M1-A15 인계 후 시험. 실제 공격 기록은 11/02</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="70" customHeight="1">
@@ -9784,13 +9817,13 @@
         <x:v>M5</x:v>
       </x:c>
       <x:c r="E132" s="75" t="n">
-        <x:v>46330</x:v>
+        <x:v>46331</x:v>
       </x:c>
       <x:c r="F132" s="75" t="n">
         <x:v>46331</x:v>
       </x:c>
       <x:c r="G132" s="74" t="str">
-        <x:v>M5-T01</x:v>
+        <x:v>M5-T01, M3-T02</x:v>
       </x:c>
       <x:c r="H132" s="74" t="str">
         <x:v>실제 적용 결과·정상 업무 유지·롤백</x:v>
@@ -9805,7 +9838,7 @@
         <x:v>조정안</x:v>
       </x:c>
       <x:c r="L132" s="74" t="str">
-        <x:v>실측 효과를 확인. 도구 설치/정책 입력만으로 효과 판정 금지</x:v>
+        <x:v>M3가 UTM3 개선 적용을 완료한 뒤 M5가 같은 조건으로 확인. M3 적용 결과·시각을 인계받고 정상 업무도 확인</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="70" customHeight="1">
@@ -9936,7 +9969,7 @@
         <x:v>M3</x:v>
       </x:c>
       <x:c r="E136" s="75" t="n">
-        <x:v>46331</x:v>
+        <x:v>46335</x:v>
       </x:c>
       <x:c r="F136" s="75" t="n">
         <x:v>46336</x:v>
@@ -9957,7 +9990,7 @@
         <x:v>미확인</x:v>
       </x:c>
       <x:c r="L136" s="74" t="str">
-        <x:v>ESXi Host 1대는 전체 Host HA가 아님. Nginx B/VIP는 자원·남은 작업 시간 판정 후 적용</x:v>
+        <x:v>11/05–06 시험 절차·대상·복구 준비, 11/09–10 실제 노드 중단·복구 시험. ESXi Host 1대의 전체 Host HA는 아님. Nginx B/VIP 적용 여부는 별도 확인</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="70" customHeight="1">
@@ -10158,7 +10191,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d10e65ebc0d4e34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc298bcad526d4b33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10330,7 +10363,7 @@
         <x:v>H04</x:v>
       </x:c>
       <x:c r="B9" s="74" t="str">
-        <x:v>10/29</x:v>
+        <x:v>10/30</x:v>
       </x:c>
       <x:c r="C9" s="74" t="str">
         <x:v>M1·M3</x:v>
@@ -10339,7 +10372,7 @@
         <x:v>M5</x:v>
       </x:c>
       <x:c r="E9" s="74" t="str">
-        <x:v>일반 라우팅·격리 Test DB·원 출발지 확인</x:v>
+        <x:v>일반 라우팅·격리 Test DB·출발지 확인 결과</x:v>
       </x:c>
       <x:c r="F9" s="74" t="str">
         <x:v>M1-A15 / M3-A10</x:v>
@@ -10348,7 +10381,7 @@
         <x:v>M5-A05 / M5-S01</x:v>
       </x:c>
       <x:c r="H9" s="74" t="str">
-        <x:v>S05는 Store/AI 완료를 기다리지 않음</x:v>
+        <x:v>10/30 경로 인계 후 M5 시험. S05는 Store/AI 완료와 독립</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="70" customHeight="1">
@@ -10694,6 +10727,29 @@
       </x:c>
       <x:c r="G28" s="91" t="str">
         <x:v>Issue 번호·체크·댓글 보존. 증거 없으면 완료로 승격하지 않음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="90" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B29" s="91" t="str">
+        <x:v>일정 점검</x:v>
+      </x:c>
+      <x:c r="C29" s="91" t="str">
+        <x:v>인계표·상세 일정 일부 불일치</x:v>
+      </x:c>
+      <x:c r="D29" s="91" t="str">
+        <x:v>S05 경로 인계 10/30·노드 시험 11/09–10</x:v>
+      </x:c>
+      <x:c r="E29" s="91" t="str">
+        <x:v>선행 작업 완료 시점과 실제 시험 순서 정리</x:v>
+      </x:c>
+      <x:c r="F29" s="91" t="str">
+        <x:v>일정 표기 보완</x:v>
+      </x:c>
+      <x:c r="G29" s="91" t="str">
+        <x:v>정상 게시판 접속은 M1 배포 후, S05 개선 확인은 M3 정책 적용 후 수행</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>